<commit_message>
version 0.07 Features Update
</commit_message>
<xml_diff>
--- a/excel/cards.xlsx
+++ b/excel/cards.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TrumpCardGenerator\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DCE0FE-F25A-4F71-A044-512DC321C867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3194B8D-A510-4602-A058-279CE04328F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{C0820614-1D59-4E6A-90A4-49D5863D6AB1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="100">
   <si>
     <t>Subject</t>
   </si>
@@ -432,6 +432,9 @@
   </si>
   <si>
     <t>Answer</t>
+  </si>
+  <si>
+    <t>Points</t>
   </si>
 </sst>
 </file>
@@ -1266,171 +1269,231 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A47AAA8D-07ED-4758-8079-A945674D8339}">
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="67.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="40.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>97</v>
       </c>
       <c r="B1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>44</v>
       </c>
       <c r="B2" s="6">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>45</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>47</v>
       </c>
       <c r="B4" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>50</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>52</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>54</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>56</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>58</v>
       </c>
       <c r="B10" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>59</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>61</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>63</v>
       </c>
       <c r="B13" s="7">
         <v>1500</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>64</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>66</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>68</v>
       </c>
       <c r="B16" s="6">
         <v>25</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>69</v>
       </c>
       <c r="B17" s="6">
         <v>999</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>70</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>72</v>
       </c>
       <c r="B19" s="7">
         <v>3000</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>73</v>
       </c>
       <c r="B20" s="7">
         <v>1000</v>
+      </c>
+      <c r="C20" s="6">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>